<commit_message>
feat(alumnos): N° lista + codigo barras + carnet imprimible + editar/regenerar; fix dup form PANOL_TP
</commit_message>
<xml_diff>
--- a/alumnos_muestra.xlsx
+++ b/alumnos_muestra.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,11 +41,6 @@
       <b val="1"/>
       <color rgb="004338CA"/>
       <sz val="14"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -93,10 +88,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -462,19 +459,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RUT / Matrícula</t>
+          <t>N° lista</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -482,146 +477,106 @@
           <t>Nombre completo</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Curso</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>19.123.456-7</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Pérez González, Juan</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>3°A Electrónica</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>juan.perez@colegio.cl</t>
-        </is>
-      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>20.234.567-8</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Soto Riquelme, María</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>3°A Electrónica</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>19.345.678-9</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Muñoz Vidal, Carlos</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>3°B Electrónica</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>20.456.789-0</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Reyes Cárdenas, Ignacia</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>3°B Electrónica</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>19.567.890-1</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Vega Toro, Felipe</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>4°A Electrónica</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>20.678.901-2</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Cortés Pino, Camila</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>4°A Electrónica</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>19.789.012-3</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Lagos Bravo, Tomás</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>4°B Electrónica</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Sandoval Olea, Sofía</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Ramírez Díaz, Matías</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Henríquez Espinoza, Florencia</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -634,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -642,7 +597,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>PLANTILLA DE CARGA DE ALUMNOS — PanolERP</t>
         </is>
@@ -674,19 +629,19 @@
       <c r="B5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Columna A (RUT / Matrícula)</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Columna A (N° lista)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>OBLIGATORIO. Identificador único del alumno. Formatos válidos: 12.345.678-9, 12345678-9, M00123.</t>
+          <t>OBLIGATORIO. Numero del alumno en su curso (1, 2, 3...). Puede repetirse entre cursos.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Columna B (Nombre completo)</t>
         </is>
@@ -698,37 +653,29 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Columna C (Curso)</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>OBLIGATORIO. Ej: "3°A Electrónica". Si no existe en tu pañol, se crea solo.</t>
-        </is>
-      </c>
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Columna D (Email)</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Opcional. Email del estudiante o apoderado.</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>IMPORTANTE:</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Antes de subir la planilla, elige el CURSO destino en el formulario web.</t>
+        </is>
+      </c>
       <c r="B10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>REGLAS:</t>
+          <t xml:space="preserve">  • Todos los alumnos de esta planilla quedaran asignados a ese curso.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -736,7 +683,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Si el RUT ya existe → se actualizan nombre, curso y email (no se duplica).</t>
+          <t xml:space="preserve">  • Si el curso aun no existe, el sistema lo crea automaticamente.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -744,7 +691,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Si el curso no existe en tu pañol → se crea automáticamente vinculado a tu especialidad.</t>
+          <t xml:space="preserve">  • Cada alumno recibe un CODIGO DE BARRAS unico para escanear su carnet.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -752,7 +699,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • La contraseña inicial del alumno = su RUT (sin puntos ni guión).</t>
+          <t xml:space="preserve">  • Si ya existe un alumno con ese (curso, N° lista), se actualiza su nombre.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -760,7 +707,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • El alumno cambia su contraseña en el primer login.</t>
+          <t xml:space="preserve">  • La contrasena inicial del alumno = su codigo de barras.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -768,7 +715,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Solo puedes cargar alumnos en TU especialidad (la del usuario logueado).</t>
+          <t xml:space="preserve">  • Solo el panolero de tu especialidad puede subir esta planilla.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -788,7 +735,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 1°A, 1°B, 2°A, 2°B (enseñanza media)</t>
+          <t xml:space="preserve">  • 1°A, 1°B, 2°A, 2°B (formacion general)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -796,7 +743,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 3°A Electrónica, 3°B Electrónica, 4°A Electrónica, 4°B Electrónica</t>
+          <t xml:space="preserve">  • 3°A Electronica, 3°B Electronica, 4°A Electronica, 4°B Electronica</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -804,18 +751,10 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 3°A Mecánica, 3°B Mecánica, 4°A Mecánica, 4°B Mecánica</t>
+          <t xml:space="preserve">  • 3°A Mecanica, 3°B Mecanica, 4°A Mecanica, 4°B Mecanica</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Adapta los nombres según tu especialidad/área.</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>